<commit_message>
Updated Sprint review protocol and TeamProtokoll
</commit_message>
<xml_diff>
--- a/Sprint_Review_Protocol_6.xlsx
+++ b/Sprint_Review_Protocol_6.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\florian\Desktop\itp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{55A846C5-7E5E-4C15-B5F9-CA7780D0734A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{711EA959-2998-45EE-99E1-633351710D41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{5C77D34F-34C3-4D2F-849C-09193AE86D67}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="98">
   <si>
     <t>Sprint Review Protocol</t>
   </si>
@@ -170,6 +170,96 @@
     <t>Anpassung des Partikelsystems war komplizierter als erwartet</t>
   </si>
   <si>
+    <t>S4MS3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enemy Open Door Logic </t>
+  </si>
+  <si>
+    <t>Schwieriger als gedacht, da ai_Controller die Tür manchmal einfach ignoriert hat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S6MS1 </t>
+  </si>
+  <si>
+    <t>Enemy Spawnpoints</t>
+  </si>
+  <si>
+    <t>Erfrischend etwas neues zu lernen</t>
+  </si>
+  <si>
+    <t>S6MS2</t>
+  </si>
+  <si>
+    <t>Skin Anpassungen</t>
+  </si>
+  <si>
+    <t>Leider keine Zeit für die Umsetzung</t>
+  </si>
+  <si>
+    <t>S6MS3</t>
+  </si>
+  <si>
+    <t>Weitere Anpassungen im Enemy State Tree</t>
+  </si>
+  <si>
+    <t>Weniger Umgesetzt als vorerst geplant deswegen weniger Zeit in Anspruch genommen</t>
+  </si>
+  <si>
+    <t>S6SM1</t>
+  </si>
+  <si>
+    <t>Filling and designing the game</t>
+  </si>
+  <si>
+    <t>Einfache Platzierungen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S6AD1 </t>
+  </si>
+  <si>
+    <t>Erschöpfungsatmen</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Keine Probleme aufgetreten</t>
+  </si>
+  <si>
+    <t>S6AD2</t>
+  </si>
+  <si>
+    <t>Gegner Jagd-Musik</t>
+  </si>
+  <si>
+    <t>Alles gemacht, jedoch Probleme in der Level Map</t>
+  </si>
+  <si>
+    <t>S6AD3</t>
+  </si>
+  <si>
+    <t>Schritte im Belüftungsschacht</t>
+  </si>
+  <si>
+    <t>Längere Bearbeitungszeit wegen Problemen</t>
+  </si>
+  <si>
+    <t>S6AD4</t>
+  </si>
+  <si>
+    <t>Leisere Schritte beim Hocken</t>
+  </si>
+  <si>
+    <t>Ging alles problemlos</t>
+  </si>
+  <si>
+    <t>S5SH1</t>
+  </si>
+  <si>
+    <t>Beleuchtung</t>
+  </si>
+  <si>
+    <t>Länge bearbeitung durch fehlendes Wissen im Bereich Blueprints</t>
+  </si>
+  <si>
     <t>Liked</t>
   </si>
   <si>
@@ -180,6 +270,54 @@
   </si>
   <si>
     <t>Longed for</t>
+  </si>
+  <si>
+    <t>Feinabstimmung von Gameplay-Mechaniken</t>
+  </si>
+  <si>
+    <t>Dynamische Footsteps, Triggerboxen und Sound mit Fade-System</t>
+  </si>
+  <si>
+    <t>Optimierung von Blueprint-Strukturen</t>
+  </si>
+  <si>
+    <t>Adaptive Musik- und Soundsysteme für Gegner</t>
+  </si>
+  <si>
+    <t>Das Überarbeiten der Wände</t>
+  </si>
+  <si>
+    <t>Arbeiten mit Blueprints und Visual Scripting</t>
+  </si>
+  <si>
+    <t>Erfahrung im Bereich Bug-fixing in Unreal Engine</t>
+  </si>
+  <si>
+    <t>Wissen in den Bereichen Performierung und Balancing</t>
+  </si>
+  <si>
+    <t>Poster selbst erstellen</t>
+  </si>
+  <si>
+    <t>Wie man eine Spielwelt realistischer bzw. voller wirken lässt</t>
+  </si>
+  <si>
+    <t>Unterschätzung, wie leer Räume aussehen</t>
+  </si>
+  <si>
+    <t>Darstellung von Objekten realistischer gestalten</t>
+  </si>
+  <si>
+    <t>Arbeiten in einem neuen Bereich von Unreal Engine(Spawnpunkte in der Welt platzieren)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SpawnLogik und besseres Verständnis für die Interaktion zwischen Objekten in der Spielwelt und ihren Blueprints </t>
+  </si>
+  <si>
+    <t>Gute Dokumentation für randomized Spawnpoints in UnrealEngine</t>
+  </si>
+  <si>
+    <t>Bessere Unreal Engine Software stabilität, damit das Programm nicht so oft abstürzt und mein Fortschritt verloren geht</t>
   </si>
   <si>
     <t>Erweiterung bestehender Mechaniken im Spiel</t>
@@ -1222,134 +1360,254 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A22" s="15"/>
-      <c r="B22" s="15"/>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
+      <c r="A22" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" s="15">
+        <v>1</v>
+      </c>
+      <c r="D22" s="15">
+        <v>3</v>
+      </c>
       <c r="E22" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F22" s="13"/>
+        <v>2</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="G22" s="14"/>
-      <c r="H22" s="16"/>
+      <c r="H22" s="16" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="23" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A23" s="15"/>
-      <c r="B23" s="16"/>
-      <c r="C23" s="15"/>
-      <c r="D23" s="15"/>
+      <c r="A23" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="15">
+        <v>2</v>
+      </c>
+      <c r="D23" s="15">
+        <v>4</v>
+      </c>
       <c r="E23" s="5">
         <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G23" s="14"/>
+      <c r="H23" s="16" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="50.25" customHeight="1">
+      <c r="A24" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="C24" s="15">
+        <v>2</v>
+      </c>
+      <c r="D24" s="15">
         <v>0</v>
       </c>
-      <c r="F23" s="13"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="16"/>
-    </row>
-    <row r="24" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A24" s="15"/>
-      <c r="B24" s="15"/>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
       <c r="E24" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="F24" s="13"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="16"/>
+      <c r="G24" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="H24" s="16" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="25" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A25" s="15"/>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
+      <c r="A25" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" s="15">
+        <v>5</v>
+      </c>
+      <c r="D25" s="15">
+        <v>3</v>
+      </c>
       <c r="E25" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F25" s="13"/>
+        <v>-2</v>
+      </c>
+      <c r="F25" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="G25" s="14"/>
-      <c r="H25" s="16"/>
+      <c r="H25" s="16" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="26" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A26" s="15"/>
-      <c r="B26" s="15"/>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
+      <c r="A26" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" s="15">
+        <v>5</v>
+      </c>
+      <c r="D26" s="15">
+        <v>5</v>
+      </c>
       <c r="E26" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F26" s="13"/>
+      <c r="F26" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="G26" s="14"/>
-      <c r="H26" s="16"/>
+      <c r="H26" s="16" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="27" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A27" s="15"/>
-      <c r="B27" s="15"/>
-      <c r="C27" s="15"/>
-      <c r="D27" s="15"/>
+      <c r="A27" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" s="15">
+        <v>3</v>
+      </c>
+      <c r="D27" s="15">
+        <v>2</v>
+      </c>
       <c r="E27" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F27" s="13"/>
+        <v>-1</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="G27" s="14"/>
-      <c r="H27" s="16"/>
+      <c r="H27" s="16" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="28" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A28" s="15"/>
-      <c r="B28" s="15"/>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
+      <c r="A28" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="C28" s="15">
+        <v>3</v>
+      </c>
+      <c r="D28" s="15">
+        <v>3</v>
+      </c>
       <c r="E28" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F28" s="13"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="16"/>
+      <c r="G28" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="H28" s="16" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="29" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A29" s="15"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="15"/>
-      <c r="D29" s="15"/>
+      <c r="A29" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="B29" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="C29" s="15">
+        <v>3</v>
+      </c>
+      <c r="D29" s="15">
+        <v>4</v>
+      </c>
       <c r="E29" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F29" s="13"/>
+        <v>1</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="G29" s="14"/>
-      <c r="H29" s="16"/>
+      <c r="H29" s="16" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="30" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A30" s="15"/>
-      <c r="B30" s="15"/>
-      <c r="C30" s="15"/>
-      <c r="D30" s="15"/>
+      <c r="A30" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="C30" s="15">
+        <v>2</v>
+      </c>
+      <c r="D30" s="15">
+        <v>2</v>
+      </c>
       <c r="E30" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F30" s="13"/>
+      <c r="F30" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="G30" s="14"/>
-      <c r="H30" s="16"/>
+      <c r="H30" s="16" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="31" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A31" s="15"/>
-      <c r="B31" s="15"/>
-      <c r="C31" s="15"/>
-      <c r="D31" s="15"/>
+      <c r="A31" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="C31" s="15">
+        <v>3</v>
+      </c>
+      <c r="D31" s="15">
+        <v>2.5</v>
+      </c>
       <c r="E31" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F31" s="13"/>
+        <v>-0.5</v>
+      </c>
+      <c r="F31" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="G31" s="14"/>
-      <c r="H31" s="16"/>
+      <c r="H31" s="16" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="32" spans="1:8" ht="50.25" customHeight="1">
       <c r="A32" s="15"/>
@@ -1402,70 +1660,102 @@
     <row r="36" spans="1:8" ht="24.75" customHeight="1">
       <c r="B36" s="4"/>
       <c r="C36" s="9" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>46</v>
+        <v>76</v>
       </c>
       <c r="F36" s="10" t="s">
-        <v>47</v>
+        <v>77</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="69.75" customHeight="1">
       <c r="B37" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C37" s="17"/>
-      <c r="D37" s="17"/>
-      <c r="E37" s="17"/>
-      <c r="F37" s="18"/>
-    </row>
-    <row r="38" spans="1:8" ht="53.25" customHeight="1">
+      <c r="C37" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="D37" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="E37" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="F37" s="18" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="82.5" customHeight="1">
       <c r="A38"/>
       <c r="B38" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C38" s="17"/>
-      <c r="D38" s="17"/>
-      <c r="E38" s="17"/>
-      <c r="F38" s="18"/>
+      <c r="C38" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="D38" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="E38" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="F38" s="18" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="39" spans="1:8" ht="96" customHeight="1">
       <c r="B39" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C39" s="17"/>
-      <c r="D39" s="17"/>
-      <c r="E39" s="17"/>
-      <c r="F39" s="18"/>
+      <c r="C39" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="D39" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="E39" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="F39" s="18" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="40" spans="1:8" ht="133.5" customHeight="1">
       <c r="B40" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C40" s="17"/>
-      <c r="D40" s="17"/>
-      <c r="E40" s="17"/>
-      <c r="F40" s="19"/>
+      <c r="C40" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="D40" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="E40" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="F40" s="19" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="41" spans="1:8" ht="60" customHeight="1">
       <c r="B41" s="8" t="s">
         <v>13</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>48</v>
+        <v>94</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>49</v>
+        <v>95</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>50</v>
+        <v>96</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>51</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>